<commit_message>
Add Q7 transformations and descriptive analysis
</commit_message>
<xml_diff>
--- a/08_tables/q7_twfe_country_correlations_i_LS.xlsx
+++ b/08_tables/q7_twfe_country_correlations_i_LS.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,6 +446,16 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>std_twfe_LS</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>std_twfe_i</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>simple_slope</t>
         </is>
       </c>
@@ -463,7 +473,13 @@
         <v>0.5843878752776019</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8373543804952331</v>
+        <v>2.318213332948363</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.617876248859742</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.8373543804952335</v>
       </c>
     </row>
     <row r="3">
@@ -479,7 +495,13 @@
         <v>0.4796868568595204</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4778646856948364</v>
+        <v>2.171745934495637</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.180027134042958</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.4778646856948366</v>
       </c>
     </row>
     <row r="4">
@@ -495,7 +517,13 @@
         <v>0.4152058736231807</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6627410574185234</v>
+        <v>2.430031241068674</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.522409443455344</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.6627410574185235</v>
       </c>
     </row>
     <row r="5">
@@ -511,7 +539,13 @@
         <v>0.3689251987654661</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2424446641801581</v>
+        <v>1.668117755779556</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2.538355202397322</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.242444664180158</v>
       </c>
     </row>
     <row r="6">
@@ -527,6 +561,12 @@
         <v>0.2359024432482654</v>
       </c>
       <c r="D6" t="n">
+        <v>2.441015882395916</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.974052946994679</v>
+      </c>
+      <c r="F6" t="n">
         <v>0.2917052511391273</v>
       </c>
     </row>
@@ -543,7 +583,13 @@
         <v>0.1864719104597827</v>
       </c>
       <c r="D7" t="n">
-        <v>0.09809357656817036</v>
+        <v>1.278923994909921</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2.431182642198552</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.09809357656817035</v>
       </c>
     </row>
     <row r="8">
@@ -559,7 +605,13 @@
         <v>0.1777081084621944</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2224417850062921</v>
+        <v>1.832622727124982</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.464077076854049</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.2224417850062919</v>
       </c>
     </row>
     <row r="9">
@@ -575,6 +627,12 @@
         <v>0.1248192927690292</v>
       </c>
       <c r="D9" t="n">
+        <v>2.921498067419213</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.466092157962786</v>
+      </c>
+      <c r="F9" t="n">
         <v>0.2487287859912337</v>
       </c>
     </row>
@@ -591,7 +649,13 @@
         <v>0.1175306650665298</v>
       </c>
       <c r="D10" t="n">
-        <v>0.3568310000170072</v>
+        <v>2.937890388957019</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9676631550796512</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.3568310000170073</v>
       </c>
     </row>
     <row r="11">
@@ -607,6 +671,12 @@
         <v>0.06451535393105778</v>
       </c>
       <c r="D11" t="n">
+        <v>1.437370431297379</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.905462521904596</v>
+      </c>
+      <c r="F11" t="n">
         <v>0.04866664184635724</v>
       </c>
     </row>
@@ -623,7 +693,13 @@
         <v>-0.02113118234055538</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.03360581447433966</v>
+        <v>2.010226608182081</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.264021291189566</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-0.03360581447433959</v>
       </c>
     </row>
     <row r="13">
@@ -639,6 +715,12 @@
         <v>-0.1193867967532351</v>
       </c>
       <c r="D13" t="n">
+        <v>1.46974698698368</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.9237158829327381</v>
+      </c>
+      <c r="F13" t="n">
         <v>-0.189959259178915</v>
       </c>
     </row>
@@ -655,7 +737,13 @@
         <v>-0.2815675730156755</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.4790808012242177</v>
+        <v>6.151909224747851</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3.615628397962685</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-0.4790808012242179</v>
       </c>
     </row>
     <row r="15">
@@ -671,6 +759,12 @@
         <v>-0.47433245651632</v>
       </c>
       <c r="D15" t="n">
+        <v>1.208114906988624</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.883554235334497</v>
+      </c>
+      <c r="F15" t="n">
         <v>-0.3042376486091111</v>
       </c>
     </row>

</xml_diff>